<commit_message>
Update company name to 'OÜ Willipu Turism' in Excel, contact footer, and all 6 languages
https://claude.ai/code/session_01DAokWKEoiBPxSJTSGSSjnQ
</commit_message>
<xml_diff>
--- a/public/hinnakiri.xlsx
+++ b/public/hinnakiri.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
-  <si>
-    <t>Willipu OÜ — Hinnakiri</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="48">
+  <si>
+    <t>OÜ Willipu Turism — Hinnakiri</t>
   </si>
   <si>
     <t>Willipu külalisemaja ja karavanipark · Pusi küla, Alatskivi vald</t>
@@ -131,6 +131,12 @@
   </si>
   <si>
     <t>Kontakt</t>
+  </si>
+  <si>
+    <t>Ettevõte</t>
+  </si>
+  <si>
+    <t>OÜ Willipu Turism</t>
   </si>
   <si>
     <t>Telefon</t>
@@ -763,7 +769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1036,8 +1042,18 @@
       <c r="C25" s="28"/>
       <c r="D25" s="28"/>
     </row>
+    <row r="26" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A3:D3"/>
@@ -1051,6 +1067,7 @@
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B26:D26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>